<commit_message>
Remove obsolete scripts and result files from the OPERA project, including dynamic class weighting, competition augmentation, advanced preprocessing, and audio transformer scripts. Update paths in the optimized insurance script for consistency.
</commit_message>
<xml_diff>
--- a/Development/Master Log Starting 251003.xlsx
+++ b/Development/Master Log Starting 251003.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Stethoscope_Project\Development\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35CF1891-41AB-465F-BF2A-59D009C70E70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{891AB066-DBD7-4DFA-947A-34175292B679}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Main" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="345" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="366" uniqueCount="186">
   <si>
     <t>Date</t>
   </si>
@@ -755,18 +755,6 @@
     <t>DA-2</t>
   </si>
   <si>
-    <t>LayerNorm + Competition DataAug + Enhanced LDAM</t>
-  </si>
-  <si>
-    <t>0.49+ (예상)</t>
-  </si>
-  <si>
-    <t>BREAKTHROUGH: Competition-grade augmentation with LayerNorm stability. Already achieving 0.444, 0.537 in first 2 folds!</t>
-  </si>
-  <si>
-    <t>step17A_competition_augmentation</t>
-  </si>
-  <si>
     <t>Step18A</t>
   </si>
   <si>
@@ -782,12 +770,6 @@
     <t>PCA(256)+ICA(128)+FeatureSelect(400)+OutlierRemoval(10%)+SmartEnsemble(5models)+OptimizedWeighting+StableAugmentation</t>
   </si>
   <si>
-    <t>[결과]</t>
-  </si>
-  <si>
-    <t>BREAKTHROUGH: Advanced preprocessing pipeline building on Step 17A success. Multi-model ensemble with optimized weighting. Target 0.52+ for Phase 2 entry.</t>
-  </si>
-  <si>
     <t>PCA(256) + ICA(128) + Feature Selection(400) + Outlier Detection(10%) + RobustScaler</t>
   </si>
   <si>
@@ -815,9 +797,6 @@
     <t>AudioSpectrogramTransformer: OPERA→48patches + MultiHeadAttention(8heads,6layers) + CLS Token + StochasticDepth + CosineWarmup + LightAugmentation</t>
   </si>
   <si>
-    <t>PHASE 2 BREAKTHROUGH: Revolutionary transformer architecture treating OPERA features as sequential patches. Self-attention mechanism for feature relationships. Target 0.60+ achieved.</t>
-  </si>
-  <si>
     <t>Audio Spectrogram Transformer: 768→48patches(16each) + Embedding(256d) + 6Layers×8Heads + CLS Token + Positional Embeddings + Stochastic Depth</t>
   </si>
   <si>
@@ -840,6 +819,69 @@
   </si>
   <si>
     <t>Reduced intensity for transformer stability while maintaining minority boost</t>
+  </si>
+  <si>
+    <t>Basic Feature Augmentation: Mixup (α=0.3) + Gaussian Noise (σ=0.03) + Minority-biased sampling</t>
+  </si>
+  <si>
+    <t>Minority Class Focus</t>
+  </si>
+  <si>
+    <t>First-generation feature augmentation</t>
+  </si>
+  <si>
+    <t>Basic augmentation techniques used in Steps 9, 9R, 10. Foundation for competition-grade augmentation.</t>
+  </si>
+  <si>
+    <t>StandardScaler</t>
+  </si>
+  <si>
+    <t>Basic normalization</t>
+  </si>
+  <si>
+    <t>Standard preprocessing</t>
+  </si>
+  <si>
+    <t>Basic standardization used across most experiments. Mean=0, Std=1 normalization.</t>
+  </si>
+  <si>
+    <t>D:/Stethoscope_Project/Development/OPERA_Copied_from_Ubuntu/scripts/GPT/step17A_final_stable.py</t>
+  </si>
+  <si>
+    <t>LayerNorm + Competition DataAug (Mixup/CutMix/Noise/Scale/Drop/Spectral/Temporal) + Enhanced LDAM-DRW + MultiRestart Tau</t>
+  </si>
+  <si>
+    <t>BREAKTHROUGH: Competition-grade augmentation (+0.170 improvement). LayerNorm stability. Best fold 0.537. Minority class boost working. Ready for Phase 2.</t>
+  </si>
+  <si>
+    <t>Advanced preprocessing pipeline with smart ensemble. Outlier removal + dimensionality reduction. Stable performance but below target. Need strategic pivot to Phase 2.</t>
+  </si>
+  <si>
+    <t>Mixup (α=0.4) + CutMix (30%) + Adaptive Gaussian Noise + Smart Feature Scaling + Advanced Dropout + Spectral Augmentation + Temporal Shift</t>
+  </si>
+  <si>
+    <t>Minority Boost (95% vs 70%) + Adaptive Parameters + LayerNorm Stability</t>
+  </si>
+  <si>
+    <t>Competition-grade multi-technique augmentation</t>
+  </si>
+  <si>
+    <t>Proven +0.170 average improvement on OPERA features, working across multiple experiments</t>
+  </si>
+  <si>
+    <t>Smart Ensemble (5 models): LinearLDAM + DeepMLP + CosineHead + LogisticRegression + RandomForest</t>
+  </si>
+  <si>
+    <t>Optimized Weighting + Soft Voting</t>
+  </si>
+  <si>
+    <t>Multi-architecture ensemble</t>
+  </si>
+  <si>
+    <t>5-model ensemble with scipy optimization for weights. Combines PyTorch and sklearn models.</t>
+  </si>
+  <si>
+    <t>Transformer experiment: Revolutionary architecture but OPERA features unsuitable for sequential modeling. Single modality limitation confirmed. 3hrs for -0.116 vs Step17A. Multimodal fusion is the real breakthrough.</t>
   </si>
 </sst>
 </file>
@@ -955,7 +997,7 @@
     <xdr:to>
       <xdr:col>15</xdr:col>
       <xdr:colOff>438150</xdr:colOff>
-      <xdr:row>7</xdr:row>
+      <xdr:row>6</xdr:row>
       <xdr:rowOff>180975</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -1301,15 +1343,15 @@
   <cols>
     <col min="1" max="1" width="13.85546875" style="1" customWidth="1"/>
     <col min="2" max="2" width="9.85546875" style="1" customWidth="1"/>
-    <col min="3" max="3" width="109.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="118.5703125" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="20.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="20.85546875" style="1" customWidth="1"/>
     <col min="6" max="6" width="14.28515625" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="17.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="29" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="30.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="109.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="18.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="123" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="220.28515625" style="1" bestFit="1" customWidth="1"/>
     <col min="12" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
@@ -1348,7 +1390,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="30">
+    <row r="2" spans="1:11">
       <c r="A2" s="3">
         <v>20251003</v>
       </c>
@@ -1488,7 +1530,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="30">
+    <row r="6" spans="1:11">
       <c r="A6" s="3">
         <v>20251004</v>
       </c>
@@ -2293,7 +2335,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="29" spans="1:11" ht="45">
+    <row r="29" spans="1:11">
       <c r="A29" s="3">
         <v>20251005</v>
       </c>
@@ -2328,7 +2370,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="30" spans="1:11" ht="30">
+    <row r="30" spans="1:11">
       <c r="A30" s="3">
         <v>20251005</v>
       </c>
@@ -2363,7 +2405,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="31" spans="1:11" ht="30">
+    <row r="31" spans="1:11">
       <c r="A31" s="3">
         <v>20251005</v>
       </c>
@@ -2433,7 +2475,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="33" spans="1:11" ht="45">
+    <row r="33" spans="1:11" ht="30">
       <c r="A33" s="3">
         <v>20251005</v>
       </c>
@@ -2476,7 +2518,7 @@
         <v>141</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>146</v>
+        <v>173</v>
       </c>
       <c r="D34" s="1" t="s">
         <v>13</v>
@@ -2494,13 +2536,13 @@
         <v>32</v>
       </c>
       <c r="I34" s="1" t="s">
-        <v>143</v>
-      </c>
-      <c r="J34" s="1" t="s">
-        <v>144</v>
+        <v>174</v>
+      </c>
+      <c r="J34" s="1">
+        <v>0.44900000000000001</v>
       </c>
       <c r="K34" s="1" t="s">
-        <v>145</v>
+        <v>175</v>
       </c>
     </row>
     <row r="35" spans="1:11">
@@ -2508,19 +2550,19 @@
         <v>20251006</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="E35" s="1" t="s">
         <v>142</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="G35" s="1" t="s">
         <v>5</v>
@@ -2529,13 +2571,13 @@
         <v>32</v>
       </c>
       <c r="I35" s="1" t="s">
-        <v>151</v>
-      </c>
-      <c r="J35" s="1" t="s">
-        <v>152</v>
+        <v>147</v>
+      </c>
+      <c r="J35" s="1">
+        <v>0.42199999999999999</v>
       </c>
       <c r="K35" s="1" t="s">
-        <v>153</v>
+        <v>176</v>
       </c>
     </row>
     <row r="36" spans="1:11">
@@ -2543,16 +2585,16 @@
         <v>20251006</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>158</v>
+        <v>152</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="F36" s="1" t="s">
         <v>15</v>
@@ -2564,13 +2606,13 @@
         <v>32</v>
       </c>
       <c r="I36" s="1" t="s">
-        <v>162</v>
-      </c>
-      <c r="J36" s="1" t="s">
-        <v>152</v>
+        <v>156</v>
+      </c>
+      <c r="J36" s="1">
+        <v>0.33300000000000002</v>
       </c>
       <c r="K36" s="1" t="s">
-        <v>163</v>
+        <v>185</v>
       </c>
     </row>
   </sheetData>
@@ -2580,14 +2622,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{12FAC5A7-032D-4B9D-85C9-8F50B46B4059}">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="5.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="59.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="89.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="41.7109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="41" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="70.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="95.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -2605,26 +2647,68 @@
       <c r="A2" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
+      <c r="B2" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>168</v>
+      </c>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
+        <v>155</v>
+      </c>
+      <c r="B3" t="s">
         <v>161</v>
       </c>
-      <c r="B3" t="s">
-        <v>168</v>
-      </c>
       <c r="C3" t="s">
-        <v>169</v>
+        <v>162</v>
       </c>
       <c r="D3" t="s">
-        <v>170</v>
+        <v>163</v>
       </c>
       <c r="E3" t="s">
-        <v>171</v>
+        <v>164</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" t="s">
+        <v>142</v>
+      </c>
+      <c r="B4" t="s">
+        <v>177</v>
+      </c>
+      <c r="C4" t="s">
+        <v>178</v>
+      </c>
+      <c r="D4" t="s">
+        <v>179</v>
+      </c>
+      <c r="E4" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5" t="s">
+        <v>155</v>
+      </c>
+      <c r="B5" t="s">
+        <v>161</v>
+      </c>
+      <c r="C5" t="s">
+        <v>162</v>
+      </c>
+      <c r="D5" t="s">
+        <v>163</v>
+      </c>
+      <c r="E5" t="s">
+        <v>164</v>
       </c>
     </row>
   </sheetData>
@@ -2671,11 +2755,11 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF38281E-CC9A-4E65-BDB5-80FEF9C10A74}">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="4.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="26.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="138" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="16.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="5.7109375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="53" customWidth="1"/>
@@ -2715,19 +2799,36 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
+        <v>145</v>
+      </c>
+      <c r="B3" t="s">
+        <v>181</v>
+      </c>
+      <c r="C3" t="s">
+        <v>182</v>
+      </c>
+      <c r="D3" t="s">
+        <v>183</v>
+      </c>
+      <c r="E3" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" t="s">
+        <v>154</v>
+      </c>
+      <c r="B4" t="s">
+        <v>157</v>
+      </c>
+      <c r="C4" t="s">
+        <v>158</v>
+      </c>
+      <c r="D4" t="s">
+        <v>159</v>
+      </c>
+      <c r="E4" t="s">
         <v>160</v>
-      </c>
-      <c r="B3" t="s">
-        <v>164</v>
-      </c>
-      <c r="C3" t="s">
-        <v>165</v>
-      </c>
-      <c r="D3" t="s">
-        <v>166</v>
-      </c>
-      <c r="E3" t="s">
-        <v>167</v>
       </c>
     </row>
   </sheetData>
@@ -2738,11 +2839,11 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28B08125-944C-452C-8E56-38E54A2D5E94}">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="5" style="7" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15" style="7" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="78" style="7" bestFit="1" customWidth="1"/>
     <col min="3" max="4" width="15.42578125" style="7" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="56.7109375" style="7" customWidth="1"/>
     <col min="6" max="16384" width="9.140625" style="7"/>
@@ -2765,21 +2866,38 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:5" ht="30">
       <c r="A2" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>171</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="45">
+      <c r="A3" s="6" t="s">
+        <v>146</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>149</v>
+      </c>
+      <c r="D3" s="6" t="s">
         <v>150</v>
       </c>
-      <c r="B2" s="6" t="s">
-        <v>154</v>
-      </c>
-      <c r="C2" s="6" t="s">
-        <v>155</v>
-      </c>
-      <c r="D2" s="6" t="s">
-        <v>156</v>
-      </c>
-      <c r="E2" s="6" t="s">
-        <v>157</v>
+      <c r="E3" s="6" t="s">
+        <v>151</v>
       </c>
     </row>
   </sheetData>

</xml_diff>